<commit_message>
Update angularidad and terrones excel templates
</commit_message>
<xml_diff>
--- a/app/templates/Template_Terrones_Fino_Grueso.xlsx
+++ b/app/templates/Template_Terrones_Fino_Grueso.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2A1E73-BC43-4167-AA46-FBD9EFC81643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15AA3DA-40EA-420A-91C1-56490EA457E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -219,7 +219,7 @@
     <numFmt numFmtId="169" formatCode="&quot;CERTIFICADO N°&quot;000&quot;-20 AG06&quot;"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -343,13 +343,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
@@ -635,7 +628,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -852,11 +845,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -887,15 +880,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -912,10 +901,10 @@
       <alignment vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -957,6 +946,65 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="12" fontId="12" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -990,75 +1038,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="12" fontId="12" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1975,35 +1964,35 @@
       <c r="I6" s="18"/>
     </row>
     <row r="7" spans="1:22" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="119" t="s">
+      <c r="A7" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="119"/>
-      <c r="C7" s="119"/>
-      <c r="D7" s="119"/>
-      <c r="E7" s="119"/>
-      <c r="F7" s="119"/>
-      <c r="G7" s="119"/>
-      <c r="H7" s="119"/>
-      <c r="I7" s="119"/>
+      <c r="B7" s="115"/>
+      <c r="C7" s="115"/>
+      <c r="D7" s="115"/>
+      <c r="E7" s="115"/>
+      <c r="F7" s="115"/>
+      <c r="G7" s="115"/>
+      <c r="H7" s="115"/>
+      <c r="I7" s="115"/>
     </row>
     <row r="8" spans="1:22" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="120" t="s">
+      <c r="A8" s="116" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="120"/>
-      <c r="C8" s="120"/>
-      <c r="D8" s="120"/>
-      <c r="E8" s="120"/>
-      <c r="F8" s="120"/>
-      <c r="G8" s="120"/>
-      <c r="H8" s="120"/>
-      <c r="I8" s="120"/>
-      <c r="Q8" s="121"/>
-      <c r="R8" s="121"/>
-      <c r="S8" s="121"/>
-      <c r="T8" s="121"/>
-      <c r="U8" s="121"/>
+      <c r="B8" s="116"/>
+      <c r="C8" s="116"/>
+      <c r="D8" s="116"/>
+      <c r="E8" s="116"/>
+      <c r="F8" s="116"/>
+      <c r="G8" s="116"/>
+      <c r="H8" s="116"/>
+      <c r="I8" s="116"/>
+      <c r="Q8" s="117"/>
+      <c r="R8" s="117"/>
+      <c r="S8" s="117"/>
+      <c r="T8" s="117"/>
+      <c r="U8" s="117"/>
       <c r="V8" s="29"/>
     </row>
     <row r="9" spans="1:22" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -2016,27 +2005,27 @@
       <c r="H9" s="27"/>
       <c r="I9" s="27"/>
       <c r="L9"/>
-      <c r="Q9" s="121"/>
-      <c r="R9" s="121"/>
-      <c r="S9" s="121"/>
-      <c r="T9" s="121"/>
-      <c r="U9" s="121"/>
+      <c r="Q9" s="117"/>
+      <c r="R9" s="117"/>
+      <c r="S9" s="117"/>
+      <c r="T9" s="117"/>
+      <c r="U9" s="117"/>
       <c r="V9" s="29"/>
     </row>
     <row r="10" spans="1:22" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="127" t="s">
+      <c r="B10" s="103" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="128"/>
-      <c r="D10" s="127" t="s">
+      <c r="C10" s="104"/>
+      <c r="D10" s="103" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="128"/>
-      <c r="F10" s="127" t="s">
+      <c r="E10" s="104"/>
+      <c r="F10" s="103" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="128"/>
-      <c r="H10" s="129" t="s">
+      <c r="G10" s="104"/>
+      <c r="H10" s="101" t="s">
         <v>53</v>
       </c>
       <c r="I10"/>
@@ -2044,13 +2033,13 @@
       <c r="L10" s="17"/>
     </row>
     <row r="11" spans="1:22" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="127"/>
-      <c r="C11" s="128"/>
-      <c r="D11" s="127"/>
-      <c r="E11" s="128"/>
-      <c r="F11" s="127"/>
-      <c r="G11" s="128"/>
-      <c r="H11" s="129"/>
+      <c r="B11" s="103"/>
+      <c r="C11" s="104"/>
+      <c r="D11" s="103"/>
+      <c r="E11" s="104"/>
+      <c r="F11" s="103"/>
+      <c r="G11" s="104"/>
+      <c r="H11" s="101"/>
       <c r="I11"/>
       <c r="K11" s="17"/>
       <c r="L11" s="17"/>
@@ -2060,36 +2049,36 @@
     <row r="12" spans="1:22" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K12" s="17"/>
       <c r="L12" s="17"/>
-      <c r="N12" s="122"/>
-      <c r="O12" s="122"/>
+      <c r="N12" s="105"/>
+      <c r="O12" s="105"/>
     </row>
     <row r="13" spans="1:22" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="103" t="s">
+      <c r="A13" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="104"/>
-      <c r="C13" s="104"/>
-      <c r="D13" s="104"/>
-      <c r="E13" s="104"/>
-      <c r="F13" s="104"/>
-      <c r="G13" s="104"/>
-      <c r="H13" s="104"/>
-      <c r="I13" s="105"/>
+      <c r="B13" s="120"/>
+      <c r="C13" s="120"/>
+      <c r="D13" s="120"/>
+      <c r="E13" s="120"/>
+      <c r="F13" s="120"/>
+      <c r="G13" s="120"/>
+      <c r="H13" s="120"/>
+      <c r="I13" s="121"/>
       <c r="J13" s="17"/>
       <c r="K13" s="17"/>
     </row>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="106" t="s">
+      <c r="A14" s="122" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="107"/>
-      <c r="C14" s="107"/>
-      <c r="D14" s="107"/>
-      <c r="E14" s="107"/>
-      <c r="F14" s="107"/>
-      <c r="G14" s="107"/>
-      <c r="H14" s="107"/>
-      <c r="I14" s="108"/>
+      <c r="B14" s="123"/>
+      <c r="C14" s="123"/>
+      <c r="D14" s="123"/>
+      <c r="E14" s="123"/>
+      <c r="F14" s="123"/>
+      <c r="G14" s="123"/>
+      <c r="H14" s="123"/>
+      <c r="I14" s="124"/>
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
     </row>
@@ -2106,37 +2095,37 @@
       <c r="K15" s="17"/>
     </row>
     <row r="16" spans="1:22" ht="19.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="111" t="s">
+      <c r="B16" s="110" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="112"/>
-      <c r="D16" s="112"/>
-      <c r="E16" s="112"/>
-      <c r="F16" s="112"/>
-      <c r="G16" s="112"/>
-      <c r="H16" s="113"/>
+      <c r="C16" s="111"/>
+      <c r="D16" s="111"/>
+      <c r="E16" s="111"/>
+      <c r="F16" s="111"/>
+      <c r="G16" s="111"/>
+      <c r="H16" s="112"/>
       <c r="I16" s="30"/>
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
     </row>
     <row r="17" spans="1:19" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="114" t="s">
+      <c r="B17" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="115"/>
-      <c r="D17" s="94" t="s">
+      <c r="C17" s="108"/>
+      <c r="D17" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="94" t="s">
+      <c r="E17" s="93" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="94" t="s">
+      <c r="F17" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="G17" s="95" t="s">
+      <c r="G17" s="94" t="s">
         <v>24</v>
       </c>
-      <c r="H17" s="95" t="s">
+      <c r="H17" s="94" t="s">
         <v>25</v>
       </c>
       <c r="I17" s="30"/>
@@ -2150,19 +2139,19 @@
       <c r="C18" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="84" t="s">
+      <c r="D18" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="84" t="s">
+      <c r="E18" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="F18" s="84" t="s">
+      <c r="F18" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="G18" s="96" t="s">
+      <c r="G18" s="95" t="s">
         <v>39</v>
       </c>
-      <c r="H18" s="96" t="s">
+      <c r="H18" s="95" t="s">
         <v>40</v>
       </c>
       <c r="I18" s="30"/>
@@ -2170,77 +2159,77 @@
       <c r="K18" s="17"/>
     </row>
     <row r="19" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="124">
+      <c r="B19" s="113">
         <v>1.5</v>
       </c>
-      <c r="C19" s="125"/>
+      <c r="C19" s="114"/>
       <c r="D19" s="79"/>
-      <c r="E19" s="130"/>
-      <c r="F19" s="130"/>
-      <c r="G19" s="97"/>
-      <c r="H19" s="97"/>
+      <c r="E19" s="102"/>
+      <c r="F19" s="102"/>
+      <c r="G19" s="96"/>
+      <c r="H19" s="96"/>
       <c r="I19" s="30"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
     </row>
     <row r="20" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="86">
+      <c r="B20" s="85">
         <v>1.5</v>
       </c>
-      <c r="C20" s="86">
+      <c r="C20" s="85">
         <v>0.75</v>
       </c>
       <c r="D20" s="79"/>
-      <c r="E20" s="130"/>
-      <c r="F20" s="130"/>
-      <c r="G20" s="97"/>
-      <c r="H20" s="97"/>
+      <c r="E20" s="102"/>
+      <c r="F20" s="102"/>
+      <c r="G20" s="96"/>
+      <c r="H20" s="96"/>
       <c r="I20" s="30"/>
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
     <row r="21" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="86">
+      <c r="B21" s="85">
         <v>0.75</v>
       </c>
-      <c r="C21" s="86">
+      <c r="C21" s="85">
         <v>0.375</v>
       </c>
       <c r="D21" s="79"/>
-      <c r="E21" s="130"/>
-      <c r="F21" s="130"/>
-      <c r="G21" s="97"/>
-      <c r="H21" s="97"/>
+      <c r="E21" s="102"/>
+      <c r="F21" s="102"/>
+      <c r="G21" s="96"/>
+      <c r="H21" s="96"/>
       <c r="I21" s="30"/>
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
     <row r="22" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="86">
+      <c r="B22" s="85">
         <v>0.375</v>
       </c>
       <c r="C22" s="80" t="s">
         <v>26</v>
       </c>
       <c r="D22" s="79"/>
-      <c r="E22" s="130"/>
-      <c r="F22" s="130"/>
-      <c r="G22" s="97"/>
-      <c r="H22" s="97"/>
+      <c r="E22" s="102"/>
+      <c r="F22" s="102"/>
+      <c r="G22" s="96"/>
+      <c r="H22" s="96"/>
       <c r="I22" s="30"/>
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
     </row>
     <row r="23" spans="1:19" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="116" t="s">
+      <c r="B23" s="109" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="116"/>
-      <c r="D23" s="116"/>
-      <c r="E23" s="116"/>
-      <c r="F23" s="116"/>
-      <c r="G23" s="116"/>
-      <c r="H23" s="97"/>
+      <c r="C23" s="109"/>
+      <c r="D23" s="109"/>
+      <c r="E23" s="109"/>
+      <c r="F23" s="109"/>
+      <c r="G23" s="109"/>
+      <c r="H23" s="96"/>
       <c r="I23" s="30"/>
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
@@ -2258,37 +2247,37 @@
       <c r="K24" s="17"/>
     </row>
     <row r="25" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="111" t="s">
+      <c r="B25" s="110" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="112"/>
-      <c r="D25" s="112"/>
-      <c r="E25" s="112"/>
-      <c r="F25" s="112"/>
-      <c r="G25" s="112"/>
-      <c r="H25" s="113"/>
+      <c r="C25" s="111"/>
+      <c r="D25" s="111"/>
+      <c r="E25" s="111"/>
+      <c r="F25" s="111"/>
+      <c r="G25" s="111"/>
+      <c r="H25" s="112"/>
       <c r="I25" s="30"/>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
     </row>
     <row r="26" spans="1:19" ht="45.6" x14ac:dyDescent="0.25">
-      <c r="B26" s="114" t="s">
+      <c r="B26" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="115"/>
-      <c r="D26" s="94" t="s">
+      <c r="C26" s="108"/>
+      <c r="D26" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="94" t="s">
+      <c r="E26" s="93" t="s">
         <v>36</v>
       </c>
-      <c r="F26" s="94" t="s">
+      <c r="F26" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="G26" s="95" t="s">
+      <c r="G26" s="94" t="s">
         <v>24</v>
       </c>
-      <c r="H26" s="95" t="s">
+      <c r="H26" s="94" t="s">
         <v>25</v>
       </c>
       <c r="I26" s="30"/>
@@ -2302,19 +2291,19 @@
       <c r="C27" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="D27" s="84" t="s">
+      <c r="D27" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="E27" s="84" t="s">
+      <c r="E27" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="F27" s="84" t="s">
+      <c r="F27" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="G27" s="96" t="s">
+      <c r="G27" s="95" t="s">
         <v>39</v>
       </c>
-      <c r="H27" s="96" t="s">
+      <c r="H27" s="95" t="s">
         <v>40</v>
       </c>
       <c r="I27" s="30"/>
@@ -2329,24 +2318,24 @@
         <v>43</v>
       </c>
       <c r="D28" s="79"/>
-      <c r="E28" s="81"/>
-      <c r="F28" s="81"/>
-      <c r="G28" s="97"/>
-      <c r="H28" s="97"/>
+      <c r="E28" s="102"/>
+      <c r="F28" s="102"/>
+      <c r="G28" s="96"/>
+      <c r="H28" s="96"/>
       <c r="I28" s="30"/>
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
     </row>
     <row r="29" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="116" t="s">
+      <c r="B29" s="109" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="116"/>
-      <c r="D29" s="116"/>
-      <c r="E29" s="116"/>
-      <c r="F29" s="116"/>
-      <c r="G29" s="116"/>
-      <c r="H29" s="97"/>
+      <c r="C29" s="109"/>
+      <c r="D29" s="109"/>
+      <c r="E29" s="109"/>
+      <c r="F29" s="109"/>
+      <c r="G29" s="109"/>
+      <c r="H29" s="96"/>
       <c r="I29" s="30"/>
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
@@ -2357,24 +2346,24 @@
       <c r="D30" s="64"/>
       <c r="E30" s="65"/>
       <c r="F30" s="65"/>
-      <c r="G30" s="98"/>
-      <c r="H30" s="98"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
       <c r="I30" s="30"/>
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
     </row>
     <row r="31" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="82"/>
-      <c r="B31" s="117" t="s">
+      <c r="A31" s="81"/>
+      <c r="B31" s="127" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="117"/>
-      <c r="D31" s="117"/>
-      <c r="E31" s="117"/>
-      <c r="F31" s="101" t="s">
+      <c r="C31" s="127"/>
+      <c r="D31" s="127"/>
+      <c r="E31" s="127"/>
+      <c r="F31" s="100" t="s">
         <v>48</v>
       </c>
-      <c r="G31" s="99"/>
+      <c r="G31" s="98"/>
       <c r="H31" s="63"/>
       <c r="I31" s="58"/>
       <c r="J31" s="35"/>
@@ -2407,15 +2396,15 @@
       <c r="S32" s="42"/>
     </row>
     <row r="33" spans="1:23" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="83"/>
-      <c r="B33" s="118" t="s">
+      <c r="A33" s="82"/>
+      <c r="B33" s="128" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="118"/>
-      <c r="D33" s="118"/>
-      <c r="E33" s="118"/>
-      <c r="F33" s="118"/>
-      <c r="G33" s="87" t="s">
+      <c r="C33" s="128"/>
+      <c r="D33" s="128"/>
+      <c r="E33" s="128"/>
+      <c r="F33" s="128"/>
+      <c r="G33" s="86" t="s">
         <v>18</v>
       </c>
       <c r="H33" s="60" t="s">
@@ -2439,10 +2428,10 @@
       <c r="D34" s="78"/>
       <c r="E34" s="67"/>
       <c r="F34" s="67"/>
-      <c r="G34" s="88" t="s">
+      <c r="G34" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="H34" s="89"/>
+      <c r="H34" s="88"/>
       <c r="J34" s="44"/>
       <c r="K34" s="32"/>
       <c r="L34" s="34"/>
@@ -2461,10 +2450,10 @@
       <c r="D35" s="78"/>
       <c r="E35" s="67"/>
       <c r="F35" s="67"/>
-      <c r="G35" s="88" t="s">
+      <c r="G35" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="H35" s="89"/>
+      <c r="H35" s="88"/>
       <c r="J35" s="44"/>
       <c r="K35" s="32"/>
       <c r="L35" s="34"/>
@@ -2488,17 +2477,17 @@
       <c r="J36" s="36"/>
       <c r="K36" s="32"/>
       <c r="L36" s="34"/>
-      <c r="M36" s="109"/>
-      <c r="N36" s="109"/>
-      <c r="O36" s="109"/>
+      <c r="M36" s="125"/>
+      <c r="N36" s="125"/>
+      <c r="O36" s="125"/>
       <c r="P36" s="47"/>
       <c r="Q36" s="47"/>
-      <c r="R36" s="109"/>
-      <c r="S36" s="109"/>
+      <c r="R36" s="125"/>
+      <c r="S36" s="125"/>
       <c r="T36" s="47"/>
-      <c r="U36" s="123"/>
-      <c r="V36" s="123"/>
-      <c r="W36" s="123"/>
+      <c r="U36" s="106"/>
+      <c r="V36" s="106"/>
+      <c r="W36" s="106"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B37" s="66"/>
@@ -2520,9 +2509,9 @@
       <c r="R37" s="47"/>
       <c r="S37" s="47"/>
       <c r="T37" s="47"/>
-      <c r="U37" s="123"/>
-      <c r="V37" s="123"/>
-      <c r="W37" s="123"/>
+      <c r="U37" s="106"/>
+      <c r="V37" s="106"/>
+      <c r="W37" s="106"/>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B38" s="77"/>
@@ -2573,16 +2562,16 @@
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="64"/>
-      <c r="B40" s="100" t="s">
+      <c r="B40" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="90"/>
-      <c r="D40" s="91"/>
-      <c r="E40" s="92"/>
-      <c r="F40" s="92"/>
-      <c r="G40" s="92"/>
-      <c r="H40" s="92"/>
-      <c r="I40" s="93"/>
+      <c r="C40" s="89"/>
+      <c r="D40" s="90"/>
+      <c r="E40" s="91"/>
+      <c r="F40" s="91"/>
+      <c r="G40" s="91"/>
+      <c r="H40" s="91"/>
+      <c r="I40" s="92"/>
       <c r="K40" s="32"/>
       <c r="L40" s="34"/>
       <c r="M40" s="48"/>
@@ -2597,8 +2586,8 @@
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A41" s="64"/>
-      <c r="B41" s="110"/>
-      <c r="C41" s="110"/>
+      <c r="B41" s="126"/>
+      <c r="C41" s="126"/>
       <c r="D41" s="73"/>
       <c r="E41" s="74"/>
       <c r="F41" s="74"/>
@@ -2631,7 +2620,7 @@
       <c r="W42" s="39"/>
     </row>
     <row r="43" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="85"/>
+      <c r="A43" s="84"/>
       <c r="K43" s="17"/>
       <c r="L43" s="34"/>
       <c r="M43" s="48"/>
@@ -2726,17 +2715,17 @@
     </row>
     <row r="49" spans="1:9" ht="13.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="102" t="s">
+      <c r="A50" s="118" t="s">
         <v>49</v>
       </c>
-      <c r="B50" s="102"/>
-      <c r="C50" s="102"/>
-      <c r="D50" s="102"/>
-      <c r="E50" s="102"/>
-      <c r="F50" s="102"/>
-      <c r="G50" s="102"/>
-      <c r="H50" s="102"/>
-      <c r="I50" s="102"/>
+      <c r="B50" s="118"/>
+      <c r="C50" s="118"/>
+      <c r="D50" s="118"/>
+      <c r="E50" s="118"/>
+      <c r="F50" s="118"/>
+      <c r="G50" s="118"/>
+      <c r="H50" s="118"/>
+      <c r="I50" s="118"/>
     </row>
     <row r="51" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="52" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2748,24 +2737,6 @@
     <protectedRange sqref="D25 C26" name="Rango3_3_1_1_1_1_1_1_1_1_1"/>
   </protectedRanges>
   <mergeCells count="29">
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="U36:W37"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="T9:U9"/>
-    <mergeCell ref="Q8:S8"/>
-    <mergeCell ref="Q9:S9"/>
     <mergeCell ref="A50:I50"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A14:I14"/>
@@ -2777,6 +2748,24 @@
     <mergeCell ref="B29:G29"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B33:F33"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="T9:U9"/>
+    <mergeCell ref="Q8:S8"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="U36:W37"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -2802,10 +2791,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="126"/>
+      <c r="B2" s="129"/>
       <c r="C2" s="8" t="s">
         <v>10</v>
       </c>

</xml_diff>